<commit_message>
product buy page update
</commit_message>
<xml_diff>
--- a/Shopping_W_data.xlsx
+++ b/Shopping_W_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6aa8e1dd04d46e4d/Desktop/shopping_site/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_F776CC53B6A7003596CC8056306D9B931B3C4078" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17578B1F-6157-4E82-9E74-01A11CAFE9FD}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="11_F776CC53B6A7003596CC8056306D9B931B3C4078" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9129CB27-FA56-4DAA-AC00-624511E626C2}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="176">
   <si>
     <t>userid</t>
   </si>
@@ -531,25 +531,25 @@
     <t>date</t>
   </si>
   <si>
-    <t>action</t>
-  </si>
-  <si>
     <t>product_id</t>
   </si>
   <si>
     <t>qty</t>
   </si>
   <si>
-    <t>UI003</t>
-  </si>
-  <si>
     <t>Yogi</t>
   </si>
   <si>
-    <t>ab.c@gmail.com</t>
-  </si>
-  <si>
     <t>a</t>
+  </si>
+  <si>
+    <t>.@gmail</t>
+  </si>
+  <si>
+    <t>size</t>
+  </si>
+  <si>
+    <t>m</t>
   </si>
 </sst>
 </file>
@@ -613,7 +613,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -624,6 +624,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3135,7 +3136,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="19.81640625" customWidth="1"/>
@@ -3171,30 +3172,30 @@
     </row>
     <row r="3" spans="1:4" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>171</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
+        <v>171</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>173</v>
       </c>
       <c r="D3" t="s">
-        <v>7</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>172</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>174</v>
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>175</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="12.5" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3205,11 +3206,10 @@
     <row r="10" spans="1:4" ht="12.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="11" spans="1:4" ht="12.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="12" spans="1:4" ht="12.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:4" ht="12.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" xr:uid="{A8CCB46B-59F7-4D08-97E7-7AAC6D55EAC7}"/>
+    <hyperlink ref="C3" r:id="rId1" xr:uid="{A8CCB46B-59F7-4D08-97E7-7AAC6D55EAC7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3220,8 +3220,11 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="13.1796875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
@@ -3237,7 +3240,24 @@
         <v>170</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>171</v>
+        <v>174</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="8">
+        <v>46218</v>
+      </c>
+      <c r="C2">
+        <v>11049</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>